<commit_message>
bootcamp certificate generation added
</commit_message>
<xml_diff>
--- a/Certificate-subhro-tech/data.xlsx
+++ b/Certificate-subhro-tech/data.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="69">
   <si>
     <t>Email</t>
   </si>
@@ -43,6 +43,189 @@
   </si>
   <si>
     <t>https://subhrotech.com</t>
+  </si>
+  <si>
+    <t>aditya.25scs1003000525@iilm.edu</t>
+  </si>
+  <si>
+    <t>depanshukumar03@gmail.com</t>
+  </si>
+  <si>
+    <t>adityaraj01107@gmail.com</t>
+  </si>
+  <si>
+    <t>tanuj.25soe1005003540@iilm.edu</t>
+  </si>
+  <si>
+    <t>akshansh.25scs1003001290@iilm.edu</t>
+  </si>
+  <si>
+    <t>sahil080805@gmail.com</t>
+  </si>
+  <si>
+    <t>mrajput24679@gmail.com</t>
+  </si>
+  <si>
+    <t>abhikushwaha909122@gmail.com</t>
+  </si>
+  <si>
+    <t>tannu.25scs1003000445@iilm.edu</t>
+  </si>
+  <si>
+    <t>alokranjan32878@gmail.com</t>
+  </si>
+  <si>
+    <t>arnav.25scs1003001276@iilm.edu</t>
+  </si>
+  <si>
+    <t>cstrider001@gmail.com</t>
+  </si>
+  <si>
+    <t>harsh.25scs1003001178@iilm.edu</t>
+  </si>
+  <si>
+    <t>khandelwalpratap@gmail.com</t>
+  </si>
+  <si>
+    <t>yuvrajthegreat07@gmail.com</t>
+  </si>
+  <si>
+    <t>aryanrajar112244@gmail.com</t>
+  </si>
+  <si>
+    <t>er9akj@gmail.com</t>
+  </si>
+  <si>
+    <t>legendrohit098@gmail.com</t>
+  </si>
+  <si>
+    <t>vidisha.25scs1003002904@iilm.edu</t>
+  </si>
+  <si>
+    <t>raushankr5080@gmail.com</t>
+  </si>
+  <si>
+    <t>whitedevil08092006@gmail.com</t>
+  </si>
+  <si>
+    <t>mr.royalaman53@gmail.com</t>
+  </si>
+  <si>
+    <t>nisaralam8527@gmail.com</t>
+  </si>
+  <si>
+    <t>manishchaudhary980mc@gmail.com</t>
+  </si>
+  <si>
+    <t>adityanarayan1016@gmail.com</t>
+  </si>
+  <si>
+    <t>777manan11@gmail.com</t>
+  </si>
+  <si>
+    <t>manindranathu@gmail.com</t>
+  </si>
+  <si>
+    <t>raushandiwan2@gmail.com</t>
+  </si>
+  <si>
+    <t>kumari350jyoti@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aditya Kumar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dipanshu kumar </t>
+  </si>
+  <si>
+    <t>Aditya Raj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanuj Mishra </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKSHANSH KUMAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sahil Kumar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohit Rajput </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abhishek Kumar Singh </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tannu kumari </t>
+  </si>
+  <si>
+    <t>ALOK RANJAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arnav </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaitanya Sharma </t>
+  </si>
+  <si>
+    <t>Harsh Singh Panwar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pratap khandelwal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yuvraj Singh </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aryan Raj </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abhishek Kumar </t>
+  </si>
+  <si>
+    <t>Rohit kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vidisha Goel </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raushan Kumar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pushpendra Singh </t>
+  </si>
+  <si>
+    <t>Aman Kumar Pathak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nisar Alam </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manish Chaudhary </t>
+  </si>
+  <si>
+    <t>Aditya Narayan Nirmal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANAN CHITTORIA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manindra Nath Upadhyay </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jyoti kumari </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IILM UNIVERSITY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chandigarh University </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ILLM UNIVERSITY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GEC Gopalganj </t>
   </si>
 </sst>
 </file>
@@ -416,12 +599,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -451,6 +634,325 @@
       </c>
       <c r="D2" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>